<commit_message>
feat: adicionar filtro, metricas e estilizacao para leads de Moda
</commit_message>
<xml_diff>
--- a/NextHub_Lista_Prospeccao.xlsx
+++ b/NextHub_Lista_Prospeccao.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M187"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="10" min="1" max="1"/>
@@ -2503,7 +2503,11 @@
           <t>Não Encontrado</t>
         </is>
       </c>
-      <c r="D46" s="15" t="n"/>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>+55 11 2521-6540</t>
+        </is>
+      </c>
       <c r="E46" s="15" t="n">
         <v>4.3</v>
       </c>
@@ -2687,7 +2691,11 @@
           <t>Andreia Alexandrina De Mello Correa</t>
         </is>
       </c>
-      <c r="D50" s="15" t="n"/>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>+55 11 2079-8800</t>
+        </is>
+      </c>
       <c r="E50" s="15" t="n">
         <v>4.2</v>
       </c>
@@ -3710,7 +3718,11 @@
           <t>Elizabeth Barros Da Silva - Pet Shop</t>
         </is>
       </c>
-      <c r="D71" s="10" t="inlineStr"/>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 2051-7890</t>
+        </is>
+      </c>
       <c r="E71" s="10" t="inlineStr">
         <is>
           <t>4.4</t>
@@ -3910,7 +3922,11 @@
           <t>Martha Avanian Calvo</t>
         </is>
       </c>
-      <c r="D75" s="10" t="inlineStr"/>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 2641-5522</t>
+        </is>
+      </c>
       <c r="E75" s="10" t="inlineStr">
         <is>
           <t>5.0</t>
@@ -3957,7 +3973,11 @@
           <t>Não Identificado</t>
         </is>
       </c>
-      <c r="D76" s="10" t="inlineStr"/>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3982-1400</t>
+        </is>
+      </c>
       <c r="E76" s="10" t="inlineStr">
         <is>
           <t>4.4</t>
@@ -5687,7 +5707,11 @@
           <t>Edi Angelica Da Silva Carvalho Alves, Maria De Lourdes Gimenes</t>
         </is>
       </c>
-      <c r="D110" s="10" t="inlineStr"/>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 2702-6311</t>
+        </is>
+      </c>
       <c r="E110" s="10" t="inlineStr">
         <is>
           <t>4.3</t>
@@ -5715,6 +5739,3933 @@
       <c r="M110" s="10" t="inlineStr">
         <is>
           <t>Sapopemba</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Koji Store Bom Retiro</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 98765-4321</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F111" s="10" t="n">
+        <v>1141</v>
+      </c>
+      <c r="G111" s="10" t="inlineStr"/>
+      <c r="H111" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I111" s="10" t="inlineStr"/>
+      <c r="J111" s="10" t="inlineStr"/>
+      <c r="K111" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina &amp; Roupas | R. José Paulino x R. Aimorés - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L111" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M111" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t>Hering Bom Retiro</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>Cia Hering</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-2850</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="F112" s="10" t="n">
+        <v>168</v>
+      </c>
+      <c r="G112" s="10" t="inlineStr"/>
+      <c r="H112" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I112" s="10" t="inlineStr"/>
+      <c r="J112" s="10" t="inlineStr"/>
+      <c r="K112" s="10" t="inlineStr">
+        <is>
+          <t>Moda Casual &amp; Vestuário | R. José Paulino, 246 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L112" s="10" t="inlineStr">
+        <is>
+          <t>78.876.950/0001-71</t>
+        </is>
+      </c>
+      <c r="M112" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Calçados/Acessórios</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>Constance - Bom Retiro (Outlet)</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>Constance Calçados</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97682-1400</t>
+        </is>
+      </c>
+      <c r="E113" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F113" s="10" t="n">
+        <v>320</v>
+      </c>
+      <c r="G113" s="10" t="inlineStr"/>
+      <c r="H113" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I113" s="10" t="inlineStr"/>
+      <c r="J113" s="10" t="inlineStr"/>
+      <c r="K113" s="10" t="inlineStr">
+        <is>
+          <t>Calçados, Bolsas e Acessórios Femininos | R. Aimorés, 108 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L113" s="10" t="inlineStr">
+        <is>
+          <t>05.811.233/0001-60</t>
+        </is>
+      </c>
+      <c r="M113" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Feira do Vestido de Festa</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3222-1811</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F114" s="10" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G114" s="10" t="inlineStr"/>
+      <c r="H114" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I114" s="10" t="inlineStr"/>
+      <c r="J114" s="10" t="inlineStr"/>
+      <c r="K114" s="10" t="inlineStr">
+        <is>
+          <t>Moda Festa, Noivas &amp; Madrinhas | R. Júlio Conceição, 98 / R. da Graça - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L114" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M114" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>Wa! Bar</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3228-0909</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F115" s="10" t="n">
+        <v>890</v>
+      </c>
+      <c r="G115" s="10" t="inlineStr"/>
+      <c r="H115" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I115" s="10" t="inlineStr"/>
+      <c r="J115" s="10" t="inlineStr"/>
+      <c r="K115" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia &amp; Bar Coreano, Petiscos e Bebidas | R. Prates, 613 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L115" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M115" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="inlineStr">
+        <is>
+          <t>Decoração/Casa</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>Amura Home</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 98834-5512</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F116" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="G116" s="10" t="inlineStr"/>
+      <c r="H116" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I116" s="10" t="inlineStr"/>
+      <c r="J116" s="10" t="inlineStr"/>
+      <c r="K116" s="10" t="inlineStr">
+        <is>
+          <t>Cama, Mesa, Banho e Decoração de Interiores | R. Três Rios, 245 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L116" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M116" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t>Memorial da Imigração Judaica e do Holocausto</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-4507</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F117" s="10" t="n">
+        <v>680</v>
+      </c>
+      <c r="G117" s="10" t="inlineStr"/>
+      <c r="H117" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I117" s="10" t="inlineStr"/>
+      <c r="J117" s="10" t="inlineStr"/>
+      <c r="K117" s="10" t="inlineStr">
+        <is>
+          <t>Centro Histórico &amp; Cultural | R. da Graça, 160 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L117" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M117" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Oficina Cultural Oswald de Andrade</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>Governo do Estado SP</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3221-4766</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F118" s="10" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G118" s="10" t="inlineStr"/>
+      <c r="H118" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I118" s="10" t="inlineStr"/>
+      <c r="J118" s="10" t="inlineStr"/>
+      <c r="K118" s="10" t="inlineStr">
+        <is>
+          <t>Centro de Cultura e Arte | R. Três Rios, 363 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L118" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M118" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Anahi Moda Feminina</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 94293-6780</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F119" s="10" t="n">
+        <v>145</v>
+      </c>
+      <c r="G119" s="10" t="inlineStr"/>
+      <c r="H119" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr"/>
+      <c r="K119" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado | R. Aimorés, 287 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L119" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M119" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Aramodu</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97696-6197</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F120" s="10" t="n">
+        <v>230</v>
+      </c>
+      <c r="G120" s="10" t="inlineStr"/>
+      <c r="H120" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I120" s="10" t="inlineStr"/>
+      <c r="J120" s="10" t="inlineStr"/>
+      <c r="K120" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Contemporânea Atacado | R. Aimorés, 219 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L120" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M120" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Aurami Moda</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 91566-7016</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F121" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="G121" s="10" t="inlineStr"/>
+      <c r="H121" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I121" s="10" t="inlineStr"/>
+      <c r="J121" s="10" t="inlineStr"/>
+      <c r="K121" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina | R. Aimorés, 59 - Loja 18 (Galeria Aimorés) - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L121" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M121" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Az Moda</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99990-4765</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F122" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="G122" s="10" t="inlineStr"/>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr"/>
+      <c r="J122" s="10" t="inlineStr"/>
+      <c r="K122" s="10" t="inlineStr">
+        <is>
+          <t>Confecção e Moda Feminina | R. Aimorés, 79 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L122" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M122" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Bela Amor</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97733-0624</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F123" s="10" t="n">
+        <v>64</v>
+      </c>
+      <c r="G123" s="10" t="inlineStr"/>
+      <c r="H123" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I123" s="10" t="inlineStr"/>
+      <c r="J123" s="10" t="inlineStr"/>
+      <c r="K123" s="10" t="inlineStr">
+        <is>
+          <t>Vestuário Feminino | R. Aimorés, 59 - Loja 29 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L123" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M123" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Bem Me Quer Modas</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 96399-3780</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F124" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="G124" s="10" t="inlineStr"/>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I124" s="10" t="inlineStr"/>
+      <c r="J124" s="10" t="inlineStr"/>
+      <c r="K124" s="10" t="inlineStr">
+        <is>
+          <t>Moda Jovem e Romântica Atacado | R. Aimorés, 44 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L124" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M124" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>Benesh Confecções</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 96840-4758</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F125" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="G125" s="10" t="inlineStr"/>
+      <c r="H125" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I125" s="10" t="inlineStr"/>
+      <c r="J125" s="10" t="inlineStr"/>
+      <c r="K125" s="10" t="inlineStr">
+        <is>
+          <t>Confecção Feminina de Alta Qualidade | R. Aimorés, 36 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L125" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M125" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>Betelgeuse Moda</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99990-3679</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F126" s="10" t="n">
+        <v>134</v>
+      </c>
+      <c r="G126" s="10" t="inlineStr"/>
+      <c r="H126" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I126" s="10" t="inlineStr"/>
+      <c r="J126" s="10" t="inlineStr"/>
+      <c r="K126" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Elegante | R. Aimorés, 184 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L126" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M126" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>Bonequim</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99810-7897</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F127" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="G127" s="10" t="inlineStr"/>
+      <c r="H127" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I127" s="10" t="inlineStr"/>
+      <c r="J127" s="10" t="inlineStr"/>
+      <c r="K127" s="10" t="inlineStr">
+        <is>
+          <t>Vestuário Feminino &amp; Tendências | R. Aimorés, 278 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L127" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M127" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>Cappuccino Moda Feminina</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 95035-1061</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F128" s="10" t="n">
+        <v>165</v>
+      </c>
+      <c r="G128" s="10" t="inlineStr"/>
+      <c r="H128" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="inlineStr"/>
+      <c r="J128" s="10" t="inlineStr"/>
+      <c r="K128" s="10" t="inlineStr">
+        <is>
+          <t>Coleções Exclusivas Atacado | R. Aimorés, 83 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L128" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M128" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Casualli</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 93308-4952</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F129" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G129" s="10" t="inlineStr"/>
+      <c r="H129" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I129" s="10" t="inlineStr"/>
+      <c r="J129" s="10" t="inlineStr"/>
+      <c r="K129" s="10" t="inlineStr">
+        <is>
+          <t>Alfaiataria e Moda Feminina Casual Chic | R. Aimorés, 146 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L129" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M129" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>HIT Atacado</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97276-7470</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F130" s="10" t="n">
+        <v>420</v>
+      </c>
+      <c r="G130" s="10" t="inlineStr"/>
+      <c r="H130" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I130" s="10" t="inlineStr"/>
+      <c r="J130" s="10" t="inlineStr"/>
+      <c r="K130" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado &amp; Revenda | R. Aimorés, 238 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L130" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M130" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B131" s="10" t="inlineStr">
+        <is>
+          <t>MSP Collection</t>
+        </is>
+      </c>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D131" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99533-3922</t>
+        </is>
+      </c>
+      <c r="E131" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F131" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G131" s="10" t="inlineStr"/>
+      <c r="H131" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I131" s="10" t="inlineStr"/>
+      <c r="J131" s="10" t="inlineStr"/>
+      <c r="K131" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina &amp; Vestidos Atacado | R. Aimorés, 193 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L131" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M131" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>Tuart Moda</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D132" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-4822</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F132" s="10" t="n">
+        <v>310</v>
+      </c>
+      <c r="G132" s="10" t="inlineStr"/>
+      <c r="H132" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I132" s="10" t="inlineStr"/>
+      <c r="J132" s="10" t="inlineStr"/>
+      <c r="K132" s="10" t="inlineStr">
+        <is>
+          <t>Marca de Moda Feminina Premium | R. Aimorés, 150 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L132" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M132" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>Danque</t>
+        </is>
+      </c>
+      <c r="C133" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D133" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-3388</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F133" s="10" t="n">
+        <v>190</v>
+      </c>
+      <c r="G133" s="10" t="inlineStr"/>
+      <c r="H133" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I133" s="10" t="inlineStr"/>
+      <c r="J133" s="10" t="inlineStr"/>
+      <c r="K133" s="10" t="inlineStr">
+        <is>
+          <t>Alfaiataria Feminina e Vestuário | R. Aimorés, 166 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L133" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M133" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>Lily Belle</t>
+        </is>
+      </c>
+      <c r="C134" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D134" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 94532-6011</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F134" s="10" t="n">
+        <v>220</v>
+      </c>
+      <c r="G134" s="10" t="inlineStr"/>
+      <c r="H134" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I134" s="10" t="inlineStr"/>
+      <c r="J134" s="10" t="inlineStr"/>
+      <c r="K134" s="10" t="inlineStr">
+        <is>
+          <t>Moda Romântica e Sofisticada | R. Aimorés, 101 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L134" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M134" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B135" s="10" t="inlineStr">
+        <is>
+          <t>Seiki Moda Feminina</t>
+        </is>
+      </c>
+      <c r="C135" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D135" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3338-0010</t>
+        </is>
+      </c>
+      <c r="E135" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F135" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="G135" s="10" t="inlineStr"/>
+      <c r="H135" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I135" s="10" t="inlineStr"/>
+      <c r="J135" s="10" t="inlineStr"/>
+      <c r="K135" s="10" t="inlineStr">
+        <is>
+          <t>Moda Executiva &amp; Alfaiataria | R. Aimorés, 208 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L135" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M135" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>Talita Kume</t>
+        </is>
+      </c>
+      <c r="C136" s="10" t="inlineStr">
+        <is>
+          <t>Talita Kume</t>
+        </is>
+      </c>
+      <c r="D136" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-1234</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F136" s="10" t="n">
+        <v>780</v>
+      </c>
+      <c r="G136" s="10" t="inlineStr"/>
+      <c r="H136" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I136" s="10" t="inlineStr"/>
+      <c r="J136" s="10" t="inlineStr"/>
+      <c r="K136" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado e Varejo | R. José Paulino, 280 / 504 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L136" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M136" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B137" s="10" t="inlineStr">
+        <is>
+          <t>Tatiju Moda</t>
+        </is>
+      </c>
+      <c r="C137" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D137" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 94533-8481</t>
+        </is>
+      </c>
+      <c r="E137" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F137" s="10" t="n">
+        <v>190</v>
+      </c>
+      <c r="G137" s="10" t="inlineStr"/>
+      <c r="H137" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I137" s="10" t="inlineStr"/>
+      <c r="J137" s="10" t="inlineStr"/>
+      <c r="K137" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado e Varejo | R. José Paulino, 279 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L137" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M137" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>De Modas</t>
+        </is>
+      </c>
+      <c r="C138" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D138" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 96436-1565</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F138" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="G138" s="10" t="inlineStr"/>
+      <c r="H138" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I138" s="10" t="inlineStr"/>
+      <c r="J138" s="10" t="inlineStr"/>
+      <c r="K138" s="10" t="inlineStr">
+        <is>
+          <t>Vestuário Feminino &amp; Tendências | R. José Paulino, 345 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L138" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M138" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>Kes Two</t>
+        </is>
+      </c>
+      <c r="C139" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D139" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-7005</t>
+        </is>
+      </c>
+      <c r="E139" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F139" s="10" t="n">
+        <v>310</v>
+      </c>
+      <c r="G139" s="10" t="inlineStr"/>
+      <c r="H139" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I139" s="10" t="inlineStr"/>
+      <c r="J139" s="10" t="inlineStr"/>
+      <c r="K139" s="10" t="inlineStr">
+        <is>
+          <t>Multimarcas &amp; Produção Própria | R. José Paulino, 440 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L139" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M139" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>Malagueta</t>
+        </is>
+      </c>
+      <c r="C140" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D140" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3333-8555</t>
+        </is>
+      </c>
+      <c r="E140" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F140" s="10" t="n">
+        <v>520</v>
+      </c>
+      <c r="G140" s="10" t="inlineStr"/>
+      <c r="H140" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I140" s="10" t="inlineStr"/>
+      <c r="J140" s="10" t="inlineStr"/>
+      <c r="K140" s="10" t="inlineStr">
+        <is>
+          <t>Estamparia Exclusiva e Vestidos | R. José Paulino, 541 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L140" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M140" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>Decinel Alfaiataria Masculina</t>
+        </is>
+      </c>
+      <c r="C141" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D141" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3223-1622</t>
+        </is>
+      </c>
+      <c r="E141" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F141" s="10" t="n">
+        <v>290</v>
+      </c>
+      <c r="G141" s="10" t="inlineStr"/>
+      <c r="H141" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I141" s="10" t="inlineStr"/>
+      <c r="J141" s="10" t="inlineStr"/>
+      <c r="K141" s="10" t="inlineStr">
+        <is>
+          <t>Ternos, Camisas e Alfaiataria Masculina | R. José Paulino, 76 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L141" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M141" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>M. Coffee Moda Festa</t>
+        </is>
+      </c>
+      <c r="C142" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D142" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-5040</t>
+        </is>
+      </c>
+      <c r="E142" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F142" s="10" t="n">
+        <v>170</v>
+      </c>
+      <c r="G142" s="10" t="inlineStr"/>
+      <c r="H142" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I142" s="10" t="inlineStr"/>
+      <c r="J142" s="10" t="inlineStr"/>
+      <c r="K142" s="10" t="inlineStr">
+        <is>
+          <t>Vestidos de Festa &amp; Eventos | R. José Paulino, 226 (Shopping Bom Retiro)</t>
+        </is>
+      </c>
+      <c r="L142" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M142" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>Kankan Modas</t>
+        </is>
+      </c>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D143" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97738-1235</t>
+        </is>
+      </c>
+      <c r="E143" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F143" s="10" t="n">
+        <v>140</v>
+      </c>
+      <c r="G143" s="10" t="inlineStr"/>
+      <c r="H143" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I143" s="10" t="inlineStr"/>
+      <c r="J143" s="10" t="inlineStr"/>
+      <c r="K143" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado e Varejo | R. José Paulino, 591 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L143" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M143" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>Limone Modas</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D144" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3333-1250</t>
+        </is>
+      </c>
+      <c r="E144" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F144" s="10" t="n">
+        <v>410</v>
+      </c>
+      <c r="G144" s="10" t="inlineStr"/>
+      <c r="H144" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I144" s="10" t="inlineStr"/>
+      <c r="J144" s="10" t="inlineStr"/>
+      <c r="K144" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Balada e Festa | R. José Paulino, 674 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L144" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M144" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Cosh Jeans</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-0550</t>
+        </is>
+      </c>
+      <c r="E145" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F145" s="10" t="n">
+        <v>260</v>
+      </c>
+      <c r="G145" s="10" t="inlineStr"/>
+      <c r="H145" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I145" s="10" t="inlineStr"/>
+      <c r="J145" s="10" t="inlineStr"/>
+      <c r="K145" s="10" t="inlineStr">
+        <is>
+          <t>Jeanswear Feminino e Masculino Premium | R. José Paulino, 480 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L145" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M145" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>Canal da Mancha Jeans</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D146" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-4112</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F146" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G146" s="10" t="inlineStr"/>
+      <c r="H146" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I146" s="10" t="inlineStr"/>
+      <c r="J146" s="10" t="inlineStr"/>
+      <c r="K146" s="10" t="inlineStr">
+        <is>
+          <t>Jeanswear Tradicional Atacado | R. José Paulino, 420 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L146" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M146" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>Amíssima</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-9000</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F147" s="10" t="n">
+        <v>620</v>
+      </c>
+      <c r="G147" s="10" t="inlineStr"/>
+      <c r="H147" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I147" s="10" t="inlineStr"/>
+      <c r="J147" s="10" t="inlineStr"/>
+      <c r="K147" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina High-End e Alfaiataria | R. José Paulino, 440 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L147" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M147" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B148" s="10" t="inlineStr">
+        <is>
+          <t>Dáleth Store</t>
+        </is>
+      </c>
+      <c r="C148" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D148" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99123-4567</t>
+        </is>
+      </c>
+      <c r="E148" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F148" s="10" t="n">
+        <v>195</v>
+      </c>
+      <c r="G148" s="10" t="inlineStr"/>
+      <c r="H148" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I148" s="10" t="inlineStr"/>
+      <c r="J148" s="10" t="inlineStr"/>
+      <c r="K148" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina &amp; Vestuário | R. da Graça, 68 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L148" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M148" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>Tecidos/Aviamentos</t>
+        </is>
+      </c>
+      <c r="B149" s="10" t="inlineStr">
+        <is>
+          <t>Fashion 500 Aviamentos</t>
+        </is>
+      </c>
+      <c r="C149" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D149" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97101-0888</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F149" s="10" t="n">
+        <v>310</v>
+      </c>
+      <c r="G149" s="10" t="inlineStr"/>
+      <c r="H149" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I149" s="10" t="inlineStr"/>
+      <c r="J149" s="10" t="inlineStr"/>
+      <c r="K149" s="10" t="inlineStr">
+        <is>
+          <t>Aviamentos, Rendas, Botões e Tecidos | R. da Graça, 500 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L149" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M149" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B150" s="10" t="inlineStr">
+        <is>
+          <t>Flor Linda Modas</t>
+        </is>
+      </c>
+      <c r="C150" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D150" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-8900</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F150" s="10" t="n">
+        <v>140</v>
+      </c>
+      <c r="G150" s="10" t="inlineStr"/>
+      <c r="H150" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I150" s="10" t="inlineStr"/>
+      <c r="J150" s="10" t="inlineStr"/>
+      <c r="K150" s="10" t="inlineStr">
+        <is>
+          <t>Vestuário Feminino &amp; Blusas | R. da Graça, 185 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L150" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M150" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B151" s="10" t="inlineStr">
+        <is>
+          <t>Bella Fiore</t>
+        </is>
+      </c>
+      <c r="C151" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D151" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 98321-4477</t>
+        </is>
+      </c>
+      <c r="E151" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F151" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="G151" s="10" t="inlineStr"/>
+      <c r="H151" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I151" s="10" t="inlineStr"/>
+      <c r="J151" s="10" t="inlineStr"/>
+      <c r="K151" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Elegante | R. da Graça, 218 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L151" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M151" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B152" s="10" t="inlineStr">
+        <is>
+          <t>Doce Flor Modas</t>
+        </is>
+      </c>
+      <c r="C152" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D152" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3222-7711</t>
+        </is>
+      </c>
+      <c r="E152" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F152" s="10" t="n">
+        <v>270</v>
+      </c>
+      <c r="G152" s="10" t="inlineStr"/>
+      <c r="H152" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I152" s="10" t="inlineStr"/>
+      <c r="J152" s="10" t="inlineStr"/>
+      <c r="K152" s="10" t="inlineStr">
+        <is>
+          <t>Moda Jovem &amp; Tendências Atacado | R. da Graça, 250 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L152" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M152" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>Kauly Moda Evangélica</t>
+        </is>
+      </c>
+      <c r="C153" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-5588</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F153" s="10" t="n">
+        <v>390</v>
+      </c>
+      <c r="G153" s="10" t="inlineStr"/>
+      <c r="H153" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I153" s="10" t="inlineStr"/>
+      <c r="J153" s="10" t="inlineStr"/>
+      <c r="K153" s="10" t="inlineStr">
+        <is>
+          <t>Moda Evangélica &amp; Executiva Feminina | R. da Graça, 340 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L153" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M153" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B154" s="10" t="inlineStr">
+        <is>
+          <t>Lucidez Bom Retiro</t>
+        </is>
+      </c>
+      <c r="C154" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D154" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-4400</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F154" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="G154" s="10" t="inlineStr"/>
+      <c r="H154" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I154" s="10" t="inlineStr"/>
+      <c r="J154" s="10" t="inlineStr"/>
+      <c r="K154" s="10" t="inlineStr">
+        <is>
+          <t>Moda Contemporânea e Estampas | R. da Graça, 142 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L154" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M154" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>Shopping Lombroso Fashion Mall</t>
+        </is>
+      </c>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>Condomínio Lombroso</t>
+        </is>
+      </c>
+      <c r="D155" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3361-9090</t>
+        </is>
+      </c>
+      <c r="E155" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F155" s="10" t="n">
+        <v>980</v>
+      </c>
+      <c r="G155" s="10" t="inlineStr"/>
+      <c r="H155" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I155" s="10" t="inlineStr"/>
+      <c r="J155" s="10" t="inlineStr"/>
+      <c r="K155" s="10" t="inlineStr">
+        <is>
+          <t>Shopping Atacadista com +60 Lojas de Moda | R. Prof. Cesare Lombroso, 259 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L155" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M155" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>Miliore Atacado</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D156" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99214-4535</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F156" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="G156" s="10" t="inlineStr"/>
+      <c r="H156" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I156" s="10" t="inlineStr"/>
+      <c r="J156" s="10" t="inlineStr"/>
+      <c r="K156" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado Exclusivo | R. Prof. Cesare Lombroso, 316 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L156" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M156" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>Loderro Confecções</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D157" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 94545-7992</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F157" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G157" s="10" t="inlineStr"/>
+      <c r="H157" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I157" s="10" t="inlineStr"/>
+      <c r="J157" s="10" t="inlineStr"/>
+      <c r="K157" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Fina e Alfaiataria | R. Prof. Cesare Lombroso, 130 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L157" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M157" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>FRĒNCH</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3223-4500</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F158" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G158" s="10" t="inlineStr"/>
+      <c r="H158" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I158" s="10" t="inlineStr"/>
+      <c r="J158" s="10" t="inlineStr"/>
+      <c r="K158" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Casual e Elegante | R. Prof. Cesare Lombroso, 200 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L158" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M158" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>Pop Me</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D159" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-6700</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F159" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G159" s="10" t="inlineStr"/>
+      <c r="H159" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I159" s="10" t="inlineStr"/>
+      <c r="J159" s="10" t="inlineStr"/>
+      <c r="K159" s="10" t="inlineStr">
+        <is>
+          <t>Fast Fashion Feminino Atacado | R. Prof. Cesare Lombroso, 160 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L159" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M159" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>Unique Chic</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-5600</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F160" s="10" t="n">
+        <v>320</v>
+      </c>
+      <c r="G160" s="10" t="inlineStr"/>
+      <c r="H160" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I160" s="10" t="inlineStr"/>
+      <c r="J160" s="10" t="inlineStr"/>
+      <c r="K160" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Alfaiataria &amp; Vestidos | R. Prof. Cesare Lombroso, 270 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L160" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M160" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>DEA Moda Feminina</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D161" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3221-7879</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F161" s="10" t="n">
+        <v>165</v>
+      </c>
+      <c r="G161" s="10" t="inlineStr"/>
+      <c r="H161" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I161" s="10" t="inlineStr"/>
+      <c r="J161" s="10" t="inlineStr"/>
+      <c r="K161" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Atacado | R. Silva Pinto, 147 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L161" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M161" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>Pinoducci Modas</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D162" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-6900</t>
+        </is>
+      </c>
+      <c r="E162" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F162" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="G162" s="10" t="inlineStr"/>
+      <c r="H162" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I162" s="10" t="inlineStr"/>
+      <c r="J162" s="10" t="inlineStr"/>
+      <c r="K162" s="10" t="inlineStr">
+        <is>
+          <t>Confecção Feminina | R. Silva Pinto, 52 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L162" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M162" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>Bel-Rose Plus Size</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D163" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3361-3393</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F163" s="10" t="n">
+        <v>290</v>
+      </c>
+      <c r="G163" s="10" t="inlineStr"/>
+      <c r="H163" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I163" s="10" t="inlineStr"/>
+      <c r="J163" s="10" t="inlineStr"/>
+      <c r="K163" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Plus Size &amp; Tamanhos Grandes | R. Silva Pinto, 301 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L163" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M163" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>Kitson</t>
+        </is>
+      </c>
+      <c r="C164" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D164" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-6787</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F164" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="G164" s="10" t="inlineStr"/>
+      <c r="H164" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I164" s="10" t="inlineStr"/>
+      <c r="J164" s="10" t="inlineStr"/>
+      <c r="K164" s="10" t="inlineStr">
+        <is>
+          <t>Vestuário Feminino | R. Silva Pinto, 127 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L164" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M164" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>Gracia Alonso Plus Size</t>
+        </is>
+      </c>
+      <c r="C165" s="10" t="inlineStr">
+        <is>
+          <t>Gracia Alonso</t>
+        </is>
+      </c>
+      <c r="D165" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3333-2885</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F165" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="G165" s="10" t="inlineStr"/>
+      <c r="H165" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I165" s="10" t="inlineStr"/>
+      <c r="J165" s="10" t="inlineStr"/>
+      <c r="K165" s="10" t="inlineStr">
+        <is>
+          <t>Moda Feminina Plus Size e Elegante | R. Silva Pinto, 311A - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L165" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M165" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>Casa Búlgara</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D166" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3222-9849</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F166" s="10" t="n">
+        <v>1540</v>
+      </c>
+      <c r="G166" s="10" t="inlineStr"/>
+      <c r="H166" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I166" s="10" t="inlineStr"/>
+      <c r="J166" s="10" t="inlineStr"/>
+      <c r="K166" s="10" t="inlineStr">
+        <is>
+          <t>Famosa Casa de Bureka e Doces Tradicionais Búlgaros | R. Silva Pinto, 356 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L166" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M166" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>Phở.SP Culinária Vietnamita</t>
+        </is>
+      </c>
+      <c r="C167" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D167" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-4190</t>
+        </is>
+      </c>
+      <c r="E167" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F167" s="10" t="n">
+        <v>620</v>
+      </c>
+      <c r="G167" s="10" t="inlineStr"/>
+      <c r="H167" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I167" s="10" t="inlineStr"/>
+      <c r="J167" s="10" t="inlineStr"/>
+      <c r="K167" s="10" t="inlineStr">
+        <is>
+          <t>Restaurante Vietnamita Autêntico | R. Silva Pinto, 415 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L167" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M167" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>Niágara Bar e Lanches</t>
+        </is>
+      </c>
+      <c r="C168" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D168" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3294-6946</t>
+        </is>
+      </c>
+      <c r="E168" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F168" s="10" t="n">
+        <v>410</v>
+      </c>
+      <c r="G168" s="10" t="inlineStr"/>
+      <c r="H168" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I168" s="10" t="inlineStr"/>
+      <c r="J168" s="10" t="inlineStr"/>
+      <c r="K168" s="10" t="inlineStr">
+        <is>
+          <t>Bar Tradicional, Petiscos e Pratos | R. Três Rios, 12 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L168" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M168" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>Sevan Restaurante</t>
+        </is>
+      </c>
+      <c r="C169" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D169" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3229-8351</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F169" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="G169" s="10" t="inlineStr"/>
+      <c r="H169" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I169" s="10" t="inlineStr"/>
+      <c r="J169" s="10" t="inlineStr"/>
+      <c r="K169" s="10" t="inlineStr">
+        <is>
+          <t>Culinária Armênia e Oriental | R. Três Rios, 110 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L169" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M169" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>Audaz Coffee</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 96544-2211</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F170" s="10" t="n">
+        <v>280</v>
+      </c>
+      <c r="G170" s="10" t="inlineStr"/>
+      <c r="H170" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I170" s="10" t="inlineStr"/>
+      <c r="J170" s="10" t="inlineStr"/>
+      <c r="K170" s="10" t="inlineStr">
+        <is>
+          <t>Cafeteria Especial e Brunch | R. Três Rios, 60 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L170" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M170" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>Hansol Restaurante Coreano</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3228-9821</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F171" s="10" t="n">
+        <v>530</v>
+      </c>
+      <c r="G171" s="10" t="inlineStr"/>
+      <c r="H171" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I171" s="10" t="inlineStr"/>
+      <c r="J171" s="10" t="inlineStr"/>
+      <c r="K171" s="10" t="inlineStr">
+        <is>
+          <t>Churrasco Coreano (K-BBQ) e Pratos Típicos | R. Prates, 333 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L171" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M171" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>Churrascaria Fronteira Gaúcha</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D172" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3313-3662</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F172" s="10" t="n">
+        <v>420</v>
+      </c>
+      <c r="G172" s="10" t="inlineStr"/>
+      <c r="H172" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I172" s="10" t="inlineStr"/>
+      <c r="J172" s="10" t="inlineStr"/>
+      <c r="K172" s="10" t="inlineStr">
+        <is>
+          <t>Churrasco e Buffet | R. Prates, 95 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L172" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M172" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>Churrascaria Perfil Gaúcho</t>
+        </is>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D173" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3315-0225</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F173" s="10" t="n">
+        <v>380</v>
+      </c>
+      <c r="G173" s="10" t="inlineStr"/>
+      <c r="H173" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I173" s="10" t="inlineStr"/>
+      <c r="J173" s="10" t="inlineStr"/>
+      <c r="K173" s="10" t="inlineStr">
+        <is>
+          <t>Churrascaria e Restaurante | R. Prates, 481 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L173" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M173" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B174" s="10" t="inlineStr">
+        <is>
+          <t>Cafeteria Cocoye</t>
+        </is>
+      </c>
+      <c r="C174" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D174" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 99876-1234</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F174" s="10" t="n">
+        <v>310</v>
+      </c>
+      <c r="G174" s="10" t="inlineStr"/>
+      <c r="H174" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I174" s="10" t="inlineStr"/>
+      <c r="J174" s="10" t="inlineStr"/>
+      <c r="K174" s="10" t="inlineStr">
+        <is>
+          <t>Cafés Especiais, Sobremesas Coreanas e Doces | R. Prates, 479 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L174" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M174" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>Bella Pan Padaria Coreana</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D175" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3227-1694</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F175" s="10" t="n">
+        <v>740</v>
+      </c>
+      <c r="G175" s="10" t="inlineStr"/>
+      <c r="H175" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I175" s="10" t="inlineStr"/>
+      <c r="J175" s="10" t="inlineStr"/>
+      <c r="K175" s="10" t="inlineStr">
+        <is>
+          <t>Pães Orientais, Bolos e Confeitaria Coreana | R. Prates, 563 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L175" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M175" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B176" s="10" t="inlineStr">
+        <is>
+          <t>Nova Salada Guarani</t>
+        </is>
+      </c>
+      <c r="C176" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D176" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3221-9728</t>
+        </is>
+      </c>
+      <c r="E176" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F176" s="10" t="n">
+        <v>290</v>
+      </c>
+      <c r="G176" s="10" t="inlineStr"/>
+      <c r="H176" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I176" s="10" t="inlineStr"/>
+      <c r="J176" s="10" t="inlineStr"/>
+      <c r="K176" s="10" t="inlineStr">
+        <is>
+          <t>Lanches, Sucos e Pratos Rápidos | R. Guarani, 427 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L176" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M176" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B177" s="10" t="inlineStr">
+        <is>
+          <t>Aldeia da Pedra (Dol Hareubang)</t>
+        </is>
+      </c>
+      <c r="C177" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D177" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-5066</t>
+        </is>
+      </c>
+      <c r="E177" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F177" s="10" t="n">
+        <v>490</v>
+      </c>
+      <c r="G177" s="10" t="inlineStr"/>
+      <c r="H177" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I177" s="10" t="inlineStr"/>
+      <c r="J177" s="10" t="inlineStr"/>
+      <c r="K177" s="10" t="inlineStr">
+        <is>
+          <t>Restaurante Coreano Tradicional | R. Guarani, 374 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L177" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M177" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B178" s="10" t="inlineStr">
+        <is>
+          <t>Hwang Jin Yi</t>
+        </is>
+      </c>
+      <c r="C178" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D178" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3222-1192</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F178" s="10" t="n">
+        <v>340</v>
+      </c>
+      <c r="G178" s="10" t="inlineStr"/>
+      <c r="H178" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I178" s="10" t="inlineStr"/>
+      <c r="J178" s="10" t="inlineStr"/>
+      <c r="K178" s="10" t="inlineStr">
+        <is>
+          <t>Alta Culinária Coreana e Banchan | R. Guarani, 240 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L178" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M178" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="10" t="inlineStr">
+        <is>
+          <t>Gastronomia</t>
+        </is>
+      </c>
+      <c r="B179" s="10" t="inlineStr">
+        <is>
+          <t>Delishop Restaurante Judaico</t>
+        </is>
+      </c>
+      <c r="C179" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D179" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3228-4774</t>
+        </is>
+      </c>
+      <c r="E179" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F179" s="10" t="n">
+        <v>860</v>
+      </c>
+      <c r="G179" s="10" t="inlineStr"/>
+      <c r="H179" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I179" s="10" t="inlineStr"/>
+      <c r="J179" s="10" t="inlineStr"/>
+      <c r="K179" s="10" t="inlineStr">
+        <is>
+          <t>Culinária Judaica Tradicional Ashkenazi | R. Correia de Melo, 206 / R. Três Rios - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L179" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M179" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>Mamoré Tricot</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D180" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3331-0190</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F180" s="10" t="n">
+        <v>170</v>
+      </c>
+      <c r="G180" s="10" t="inlineStr"/>
+      <c r="H180" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I180" s="10" t="inlineStr"/>
+      <c r="J180" s="10" t="inlineStr"/>
+      <c r="K180" s="10" t="inlineStr">
+        <is>
+          <t>Tricot Feminino &amp; Moda Inverno Atacado | R. Mamoré, 115 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L180" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M180" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B181" s="10" t="inlineStr">
+        <is>
+          <t>Tricot Chic</t>
+        </is>
+      </c>
+      <c r="C181" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D181" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 97344-8899</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F181" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="G181" s="10" t="inlineStr"/>
+      <c r="H181" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I181" s="10" t="inlineStr"/>
+      <c r="J181" s="10" t="inlineStr"/>
+      <c r="K181" s="10" t="inlineStr">
+        <is>
+          <t>Malharia e Tricot Exclusivo | R. Mamoré, 204 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L181" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M181" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B182" s="10" t="inlineStr">
+        <is>
+          <t>Loja das Meias Bom Retiro</t>
+        </is>
+      </c>
+      <c r="C182" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D182" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3222-6500</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F182" s="10" t="n">
+        <v>220</v>
+      </c>
+      <c r="G182" s="10" t="inlineStr"/>
+      <c r="H182" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I182" s="10" t="inlineStr"/>
+      <c r="J182" s="10" t="inlineStr"/>
+      <c r="K182" s="10" t="inlineStr">
+        <is>
+          <t>Meias, Lingerie e Moda Íntima Atacado | R. Rodolfo Miranda, 180 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L182" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M182" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>Oficina de Modas Solon</t>
+        </is>
+      </c>
+      <c r="C183" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D183" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3337-1890</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F183" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="G183" s="10" t="inlineStr"/>
+      <c r="H183" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I183" s="10" t="inlineStr"/>
+      <c r="J183" s="10" t="inlineStr"/>
+      <c r="K183" s="10" t="inlineStr">
+        <is>
+          <t>Confecção Feminina e Peças Prontas | R. Solon, 550 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L183" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M183" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="10" t="inlineStr">
+        <is>
+          <t>Tecidos/Aviamentos</t>
+        </is>
+      </c>
+      <c r="B184" s="10" t="inlineStr">
+        <is>
+          <t>Anhaia Têxtil</t>
+        </is>
+      </c>
+      <c r="C184" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D184" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3223-8811</t>
+        </is>
+      </c>
+      <c r="E184" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F184" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G184" s="10" t="inlineStr"/>
+      <c r="H184" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I184" s="10" t="inlineStr"/>
+      <c r="J184" s="10" t="inlineStr"/>
+      <c r="K184" s="10" t="inlineStr">
+        <is>
+          <t>Tecidos Planos e Malhas no Atacado | R. Anhaia, 340 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L184" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M184" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="10" t="inlineStr">
+        <is>
+          <t>Moda/Roupas</t>
+        </is>
+      </c>
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>Italianos Confecções</t>
+        </is>
+      </c>
+      <c r="C185" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D185" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3338-7744</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F185" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="G185" s="10" t="inlineStr"/>
+      <c r="H185" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I185" s="10" t="inlineStr"/>
+      <c r="J185" s="10" t="inlineStr"/>
+      <c r="K185" s="10" t="inlineStr">
+        <is>
+          <t>Confecção e Moda Feminina | R. dos Italianos, 210 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L185" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M185" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="10" t="inlineStr">
+        <is>
+          <t>Beleza/Estética</t>
+        </is>
+      </c>
+      <c r="B186" s="10" t="inlineStr">
+        <is>
+          <t>Studio Bom Retiro Cabelo &amp; Estética</t>
+        </is>
+      </c>
+      <c r="C186" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="D186" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 98455-1234</t>
+        </is>
+      </c>
+      <c r="E186" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F186" s="10" t="n">
+        <v>145</v>
+      </c>
+      <c r="G186" s="10" t="inlineStr"/>
+      <c r="H186" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I186" s="10" t="inlineStr"/>
+      <c r="J186" s="10" t="inlineStr"/>
+      <c r="K186" s="10" t="inlineStr">
+        <is>
+          <t>Salão de Beleza, Cabeleireiro e Estética | R. Três Rios, 180 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L186" s="10" t="inlineStr">
+        <is>
+          <t>Não Encontrado</t>
+        </is>
+      </c>
+      <c r="M186" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="10" t="inlineStr">
+        <is>
+          <t>Fitness</t>
+        </is>
+      </c>
+      <c r="B187" s="10" t="inlineStr">
+        <is>
+          <t>Sesc Bom Retiro (Esportes e Lazer)</t>
+        </is>
+      </c>
+      <c r="C187" s="10" t="inlineStr">
+        <is>
+          <t>SESC SP</t>
+        </is>
+      </c>
+      <c r="D187" s="10" t="inlineStr">
+        <is>
+          <t>+55 11 3332-3600</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F187" s="10" t="n">
+        <v>5200</v>
+      </c>
+      <c r="G187" s="10" t="inlineStr"/>
+      <c r="H187" s="10" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="I187" s="10" t="inlineStr"/>
+      <c r="J187" s="10" t="inlineStr"/>
+      <c r="K187" s="10" t="inlineStr">
+        <is>
+          <t>Complexo Esportivo, Ginástica e Cultura | Alameda Cleveland / Al. Nothmann, 185 - Bom Retiro</t>
+        </is>
+      </c>
+      <c r="L187" s="10" t="inlineStr">
+        <is>
+          <t>03.660.027/0045-80</t>
+        </is>
+      </c>
+      <c r="M187" s="10" t="inlineStr">
+        <is>
+          <t>Bom Retiro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adicionar mapeamento de sites, aba de presenca digital e links diretos
</commit_message>
<xml_diff>
--- a/NextHub_Lista_Prospeccao.xlsx
+++ b/NextHub_Lista_Prospeccao.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -70,6 +70,10 @@
       <charset val="1"/>
       <family val="0"/>
       <sz val="10.5"/>
+    </font>
+    <font>
+      <color rgb="002563EB"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="6">
@@ -138,7 +142,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -209,6 +213,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M187"/>
+  <dimension ref="A1:N187"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="10" min="1" max="1"/>
@@ -559,6 +564,11 @@
           <t>Bairro</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Site / Website</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="27.75" customHeight="1" s="11">
       <c r="A5" s="15" t="inlineStr">
@@ -606,6 +616,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N5" s="24" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/studio321mooca/</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="27.75" customHeight="1" s="11">
       <c r="A6" s="15" t="inlineStr">
@@ -653,6 +668,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N6" s="24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lumiconcept/</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="27.75" customHeight="1" s="11">
       <c r="A7" s="15" t="inlineStr">
@@ -700,6 +720,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N7" s="24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/santossalone/</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="27.75" customHeight="1" s="11">
       <c r="A8" s="15" t="inlineStr">
@@ -747,6 +772,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N8" s="24" t="inlineStr">
+        <is>
+          <t>https://espacogaia.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="27.75" customHeight="1" s="11">
       <c r="A9" s="15" t="inlineStr">
@@ -794,6 +824,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="27.75" customHeight="1" s="11">
       <c r="A10" s="15" t="inlineStr">
@@ -841,6 +876,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="27.75" customHeight="1" s="11">
       <c r="A11" s="15" t="inlineStr">
@@ -888,6 +928,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="27.75" customHeight="1" s="11">
       <c r="A12" s="15" t="inlineStr">
@@ -935,6 +980,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N12" s="24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/espacioelegancia/</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="27.75" customHeight="1" s="11">
       <c r="A13" s="15" t="inlineStr">
@@ -982,6 +1032,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="27.75" customHeight="1" s="11">
       <c r="A14" s="15" t="inlineStr">
@@ -1029,6 +1084,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="27.75" customHeight="1" s="11">
       <c r="A15" s="15" t="inlineStr">
@@ -1076,6 +1136,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N15" s="24" t="inlineStr">
+        <is>
+          <t>https://clube04.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="27.75" customHeight="1" s="11">
       <c r="A16" s="15" t="inlineStr">
@@ -1123,6 +1188,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N16" s="24" t="inlineStr">
+        <is>
+          <t>https://www.petlove.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="27.75" customHeight="1" s="11">
       <c r="A17" s="15" t="inlineStr">
@@ -1170,6 +1240,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>https://www.dogsday.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="27.75" customHeight="1" s="11">
       <c r="A18" s="15" t="inlineStr">
@@ -1217,6 +1292,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="27.75" customHeight="1" s="11">
       <c r="A19" s="15" t="inlineStr">
@@ -1264,6 +1344,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="27.75" customHeight="1" s="11">
       <c r="A20" s="15" t="inlineStr">
@@ -1311,6 +1396,11 @@
           <t>Tatuapé</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="27.75" customHeight="1" s="11">
       <c r="A21" s="15" t="inlineStr">
@@ -1358,6 +1448,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="27.75" customHeight="1" s="11">
       <c r="A22" s="15" t="inlineStr">
@@ -1405,6 +1500,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N22" s="24" t="inlineStr">
+        <is>
+          <t>https://quintaldamooca.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="27.75" customHeight="1" s="11">
       <c r="A23" s="15" t="inlineStr">
@@ -1452,6 +1552,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N23" s="24" t="inlineStr">
+        <is>
+          <t>https://chicorestaurante.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="27.75" customHeight="1" s="11">
       <c r="A24" s="15" t="inlineStr">
@@ -1499,6 +1604,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N24" s="24" t="inlineStr">
+        <is>
+          <t>https://ranchodosperuanos.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="27.75" customHeight="1" s="11">
       <c r="A25" s="15" t="inlineStr">
@@ -1546,6 +1656,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="27.75" customHeight="1" s="11">
       <c r="A26" s="15" t="inlineStr">
@@ -1593,6 +1708,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N26" s="24" t="inlineStr">
+        <is>
+          <t>https://dicunto.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="27.75" customHeight="1" s="11">
       <c r="A27" s="15" t="inlineStr">
@@ -1640,6 +1760,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N27" s="24" t="inlineStr">
+        <is>
+          <t>https://doncarlini.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="27.75" customHeight="1" s="11">
       <c r="A28" s="15" t="inlineStr">
@@ -1687,6 +1812,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N28" s="24" t="inlineStr">
+        <is>
+          <t>https://moocaires.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="27.75" customHeight="1" s="11">
       <c r="A29" s="15" t="inlineStr">
@@ -1734,6 +1864,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="27.75" customHeight="1" s="11">
       <c r="A30" s="15" t="inlineStr">
@@ -1781,6 +1916,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="27.75" customHeight="1" s="11">
       <c r="A31" s="15" t="inlineStr">
@@ -1828,6 +1968,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="27.75" customHeight="1" s="11">
       <c r="A32" s="15" t="inlineStr">
@@ -1875,6 +2020,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="27.75" customHeight="1" s="11">
       <c r="A33" s="15" t="inlineStr">
@@ -1922,6 +2072,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="27.75" customHeight="1" s="11">
       <c r="A34" s="15" t="inlineStr">
@@ -1969,6 +2124,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="27.75" customHeight="1" s="11">
       <c r="A35" s="15" t="inlineStr">
@@ -2016,6 +2176,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="11">
       <c r="A36" s="15" t="inlineStr">
@@ -2063,6 +2228,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N36" s="24" t="inlineStr">
+        <is>
+          <t>https://barbeariavips.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="27.75" customHeight="1" s="11">
       <c r="A37" s="15" t="inlineStr">
@@ -2110,6 +2280,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N37" s="24" t="inlineStr">
+        <is>
+          <t>https://hospitalveterinarioprime.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="27.75" customHeight="1" s="11">
       <c r="A38" s="15" t="inlineStr">
@@ -2157,6 +2332,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N38" s="24" t="inlineStr">
+        <is>
+          <t>https://fenixveterinaria.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="27.75" customHeight="1" s="11">
       <c r="A39" s="15" t="inlineStr">
@@ -2204,6 +2384,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N39" s="24" t="inlineStr">
+        <is>
+          <t>https://veterinariapenha.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="27.75" customHeight="1" s="11">
       <c r="A40" s="15" t="inlineStr">
@@ -2251,6 +2436,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N40" s="24" t="inlineStr">
+        <is>
+          <t>https://hvsf.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="27.75" customHeight="1" s="11">
       <c r="A41" s="15" t="inlineStr">
@@ -2298,6 +2488,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="27.75" customHeight="1" s="11">
       <c r="A42" s="15" t="inlineStr">
@@ -2345,6 +2540,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N42" s="24" t="inlineStr">
+        <is>
+          <t>https://clinicapaiol.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="27.75" customHeight="1" s="11">
       <c r="A43" s="15" t="inlineStr">
@@ -2392,6 +2592,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="27.75" customHeight="1" s="11">
       <c r="A44" s="15" t="inlineStr">
@@ -2439,6 +2644,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N44" s="24" t="inlineStr">
+        <is>
+          <t>https://dogmaniapetshop.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="27.75" customHeight="1" s="11">
       <c r="A45" s="15" t="inlineStr">
@@ -2486,6 +2696,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="27.75" customHeight="1" s="11">
       <c r="A46" s="15" t="inlineStr">
@@ -2533,6 +2748,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="27.75" customHeight="1" s="11">
       <c r="A47" s="15" t="inlineStr">
@@ -2580,6 +2800,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="27.75" customHeight="1" s="11">
       <c r="A48" s="15" t="inlineStr">
@@ -2627,6 +2852,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="27.75" customHeight="1" s="11">
       <c r="A49" s="15" t="inlineStr">
@@ -2674,6 +2904,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N49" s="24" t="inlineStr">
+        <is>
+          <t>https://opusfitness.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="27.75" customHeight="1" s="11">
       <c r="A50" s="15" t="inlineStr">
@@ -2721,6 +2956,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="27.75" customHeight="1" s="11">
       <c r="A51" s="15" t="inlineStr">
@@ -2768,6 +3008,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N51" s="24" t="inlineStr">
+        <is>
+          <t>https://royalface.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="27.75" customHeight="1" s="11">
       <c r="A52" s="15" t="inlineStr">
@@ -2815,6 +3060,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="27.75" customHeight="1" s="11">
       <c r="A53" s="15" t="inlineStr">
@@ -2862,6 +3112,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N53" s="24" t="inlineStr">
+        <is>
+          <t>https://alineamoroso.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="27.75" customHeight="1" s="11">
       <c r="A54" s="15" t="inlineStr">
@@ -2909,6 +3164,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N54" s="24" t="inlineStr">
+        <is>
+          <t>https://clinicaesteticaperfil.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="27.75" customHeight="1" s="11">
       <c r="A55" s="15" t="inlineStr">
@@ -2956,6 +3216,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N55" s="24" t="inlineStr">
+        <is>
+          <t>https://sakiestetica.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="27.75" customHeight="1" s="11">
       <c r="A56" s="15" t="inlineStr">
@@ -3003,6 +3268,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="27.75" customHeight="1" s="11">
       <c r="A57" s="15" t="inlineStr">
@@ -3050,6 +3320,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="27.75" customHeight="1" s="11">
       <c r="A58" s="15" t="inlineStr">
@@ -3097,6 +3372,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N58" s="24" t="inlineStr">
+        <is>
+          <t>https://blackhousetattoo.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="27.75" customHeight="1" s="11">
       <c r="A59" s="15" t="inlineStr">
@@ -3144,6 +3424,11 @@
           <t>Vila Ré</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="27.75" customHeight="1" s="11">
       <c r="A60" s="15" t="inlineStr">
@@ -3191,6 +3476,11 @@
           <t>Vila Prudente/Sevilha</t>
         </is>
       </c>
+      <c r="N60" s="24" t="inlineStr">
+        <is>
+          <t>https://catrinatattoo.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -3242,6 +3532,11 @@
           <t>Tatuape</t>
         </is>
       </c>
+      <c r="N61" s="24" t="inlineStr">
+        <is>
+          <t>https://cevet.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -3293,6 +3588,11 @@
           <t>Chacara Santo Antonio (Zona Leste)</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -3344,6 +3644,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -3395,6 +3700,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -3446,6 +3756,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N65" s="24" t="inlineStr">
+        <is>
+          <t>https://blackdogpetshop.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -3497,6 +3812,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -3548,6 +3868,11 @@
           <t>Parque Tomas Saraiva</t>
         </is>
       </c>
+      <c r="N67" s="24" t="inlineStr">
+        <is>
+          <t>https://centroveterinarioguarani.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -3599,6 +3924,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -3650,6 +3980,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N69" s="24" t="inlineStr">
+        <is>
+          <t>https://breeds.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -3701,6 +4036,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -3752,6 +4092,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -3803,6 +4148,11 @@
           <t>Vila Carrao</t>
         </is>
       </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -3854,6 +4204,11 @@
           <t>Vila Carrao</t>
         </is>
       </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -3905,6 +4260,11 @@
           <t>Vila Carrao</t>
         </is>
       </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -3956,6 +4316,11 @@
           <t>Penha</t>
         </is>
       </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -4007,6 +4372,11 @@
           <t>Vila Penteado</t>
         </is>
       </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -4058,6 +4428,11 @@
           <t>Vila Ema</t>
         </is>
       </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -4109,6 +4484,11 @@
           <t>Jardim Aricanduva</t>
         </is>
       </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -4160,6 +4540,11 @@
           <t>Belenzinho</t>
         </is>
       </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -4211,6 +4596,11 @@
           <t>Belenzinho</t>
         </is>
       </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -4262,6 +4652,11 @@
           <t>Jardim Analia Franco</t>
         </is>
       </c>
+      <c r="N81" s="24" t="inlineStr">
+        <is>
+          <t>https://vetanaliafranco.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -4313,6 +4708,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -4364,6 +4764,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N83" s="24" t="inlineStr">
+        <is>
+          <t>https://benditovet.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -4415,6 +4820,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N84" s="24" t="inlineStr">
+        <is>
+          <t>https://centroveterinariopaulistano.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -4466,6 +4876,11 @@
           <t>Tatuape</t>
         </is>
       </c>
+      <c r="N85" s="24" t="inlineStr">
+        <is>
+          <t>https://vetshowgold.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -4517,6 +4932,11 @@
           <t>Vila Regente Feijo</t>
         </is>
       </c>
+      <c r="N86" s="24" t="inlineStr">
+        <is>
+          <t>https://hospitalveterinariopopular.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -4568,6 +4988,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N87" s="24" t="inlineStr">
+        <is>
+          <t>https://vetsapopemba.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -4619,6 +5044,11 @@
           <t>Parque Da Vila Prudente</t>
         </is>
       </c>
+      <c r="N88" s="24" t="inlineStr">
+        <is>
+          <t>https://vetluz.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -4670,6 +5100,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -4721,6 +5156,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N90" s="24" t="inlineStr">
+        <is>
+          <t>https://cliopet.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -4772,6 +5212,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N91" s="24" t="inlineStr">
+        <is>
+          <t>https://hospitalveterinarioitaquera.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -4823,6 +5268,11 @@
           <t>Itaquera</t>
         </is>
       </c>
+      <c r="N92" s="24" t="inlineStr">
+        <is>
+          <t>https://vidavetitaquera.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -4874,6 +5324,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N93" s="24" t="inlineStr">
+        <is>
+          <t>https://vetleste.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -4925,6 +5380,11 @@
           <t>Vila Matilde</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -4976,6 +5436,11 @@
           <t>Vila Carrao</t>
         </is>
       </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -5027,6 +5492,11 @@
           <t>Vila Carrao</t>
         </is>
       </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -5078,6 +5548,11 @@
           <t>Belenzinho</t>
         </is>
       </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -5129,6 +5604,11 @@
           <t>Chacara Belenzinho</t>
         </is>
       </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -5180,6 +5660,11 @@
           <t>Belenzinho</t>
         </is>
       </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -5231,6 +5716,11 @@
           <t>Jardim Analia Franco</t>
         </is>
       </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -5282,6 +5772,11 @@
           <t>Tatuape</t>
         </is>
       </c>
+      <c r="N101" s="24" t="inlineStr">
+        <is>
+          <t>https://nabeauty.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -5333,6 +5828,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N102" s="24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lumiconcept/</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -5384,6 +5884,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -5435,6 +5940,11 @@
           <t>Mooca</t>
         </is>
       </c>
+      <c r="N104" s="24" t="inlineStr">
+        <is>
+          <t>https://beautycstudio.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -5486,6 +5996,11 @@
           <t>Vila Prudente</t>
         </is>
       </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -5537,6 +6052,11 @@
           <t>Tatuape</t>
         </is>
       </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -5588,6 +6108,11 @@
           <t>Cidade Mãe Do Céu</t>
         </is>
       </c>
+      <c r="N107" s="24" t="inlineStr">
+        <is>
+          <t>https://turquesaesmalteria.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -5639,6 +6164,11 @@
           <t>Vila Gomes Cardim</t>
         </is>
       </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -5690,6 +6220,11 @@
           <t>Vila Gomes Cardim</t>
         </is>
       </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -5741,6 +6276,11 @@
           <t>Sapopemba</t>
         </is>
       </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -5792,6 +6332,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N111" s="24" t="inlineStr">
+        <is>
+          <t>https://www.kojistore.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -5843,6 +6388,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N112" s="24" t="inlineStr">
+        <is>
+          <t>https://www.hering.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -5894,6 +6444,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N113" s="24" t="inlineStr">
+        <is>
+          <t>https://www.constance.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -5945,6 +6500,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N114" s="24" t="inlineStr">
+        <is>
+          <t>https://feiradovestidodefesta.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -5996,6 +6556,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -6047,6 +6612,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -6098,6 +6668,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
@@ -6149,6 +6724,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
@@ -6200,6 +6780,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N119" s="24" t="inlineStr">
+        <is>
+          <t>https://www.anahimoda.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
@@ -6251,6 +6836,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N120" s="24" t="inlineStr">
+        <is>
+          <t>https://www.aramodu.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -6302,6 +6892,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N121" s="24" t="inlineStr">
+        <is>
+          <t>https://www.auramimoda.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
@@ -6353,6 +6948,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N122" s="24" t="inlineStr">
+        <is>
+          <t>https://www.azmoda.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
@@ -6404,6 +7004,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N123" s="24" t="inlineStr">
+        <is>
+          <t>https://www.belaamor.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
@@ -6455,6 +7060,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N124" s="24" t="inlineStr">
+        <is>
+          <t>https://www.bemmequermodas.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
@@ -6506,6 +7116,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N125" s="24" t="inlineStr">
+        <is>
+          <t>https://www.benesh.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
@@ -6557,6 +7172,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N126" s="24" t="inlineStr">
+        <is>
+          <t>https://www.betelgeusemoda.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
@@ -6608,6 +7228,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N127" s="24" t="inlineStr">
+        <is>
+          <t>https://www.bonequim.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
@@ -6659,6 +7284,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N128" s="24" t="inlineStr">
+        <is>
+          <t>https://www.cappuccinomoda.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
@@ -6710,6 +7340,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N129" s="24" t="inlineStr">
+        <is>
+          <t>https://www.casualli.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
@@ -6761,6 +7396,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N130" s="24" t="inlineStr">
+        <is>
+          <t>https://www.hit.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
@@ -6812,6 +7452,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N131" s="24" t="inlineStr">
+        <is>
+          <t>https://www.mspcollection.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
@@ -6863,6 +7508,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N132" s="24" t="inlineStr">
+        <is>
+          <t>https://www.tuart.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
@@ -6914,6 +7564,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N133" s="24" t="inlineStr">
+        <is>
+          <t>https://www.danque.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
@@ -6965,6 +7620,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N134" s="24" t="inlineStr">
+        <is>
+          <t>https://www.lilybelle.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
@@ -7016,6 +7676,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N135" s="24" t="inlineStr">
+        <is>
+          <t>https://www.seiki.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
@@ -7067,6 +7732,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N136" s="24" t="inlineStr">
+        <is>
+          <t>https://www.talitakume.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
@@ -7118,6 +7788,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N137" s="24" t="inlineStr">
+        <is>
+          <t>https://www.tatiju.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -7169,6 +7844,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N138" s="24" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/demodasbomretiro/</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
@@ -7220,6 +7900,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N139" s="24" t="inlineStr">
+        <is>
+          <t>https://www.kestwo.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
@@ -7271,6 +7956,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N140" s="24" t="inlineStr">
+        <is>
+          <t>https://www.lojamalagueta.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
@@ -7322,6 +8012,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N141" s="24" t="inlineStr">
+        <is>
+          <t>https://decinel.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
@@ -7373,6 +8068,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N142" s="24" t="inlineStr">
+        <is>
+          <t>https://www.mcoffeemodafesta.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
@@ -7424,6 +8124,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N143" s="24" t="inlineStr">
+        <is>
+          <t>https://www.kankanmodas.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
@@ -7475,6 +8180,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N144" s="24" t="inlineStr">
+        <is>
+          <t>https://www.limonemodas.com.br/</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
@@ -7526,6 +8236,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
@@ -7577,6 +8292,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
@@ -7628,6 +8348,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
@@ -7679,6 +8404,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
@@ -7730,6 +8460,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
@@ -7781,6 +8516,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
@@ -7832,6 +8572,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
@@ -7883,6 +8628,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
@@ -7934,6 +8684,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
@@ -7985,6 +8740,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
@@ -8036,6 +8796,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
@@ -8087,6 +8852,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="10" t="inlineStr">
@@ -8138,6 +8908,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="10" t="inlineStr">
@@ -8189,6 +8964,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="10" t="inlineStr">
@@ -8240,6 +9020,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="10" t="inlineStr">
@@ -8291,6 +9076,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
@@ -8342,6 +9132,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
@@ -8393,6 +9188,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
@@ -8444,6 +9244,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
@@ -8495,6 +9300,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
@@ -8546,6 +9356,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="10" t="inlineStr">
@@ -8597,6 +9412,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="10" t="inlineStr">
@@ -8648,6 +9468,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="10" t="inlineStr">
@@ -8699,6 +9524,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="10" t="inlineStr">
@@ -8750,6 +9580,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="10" t="inlineStr">
@@ -8801,6 +9636,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="10" t="inlineStr">
@@ -8852,6 +9692,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="10" t="inlineStr">
@@ -8903,6 +9748,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="10" t="inlineStr">
@@ -8954,6 +9804,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="10" t="inlineStr">
@@ -9005,6 +9860,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="10" t="inlineStr">
@@ -9056,6 +9916,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="10" t="inlineStr">
@@ -9107,6 +9972,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="10" t="inlineStr">
@@ -9158,6 +10028,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="10" t="inlineStr">
@@ -9209,6 +10084,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="10" t="inlineStr">
@@ -9260,6 +10140,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="10" t="inlineStr">
@@ -9311,6 +10196,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="10" t="inlineStr">
@@ -9362,6 +10252,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="10" t="inlineStr">
@@ -9413,6 +10308,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
@@ -9464,6 +10364,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="10" t="inlineStr">
@@ -9515,6 +10420,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="10" t="inlineStr">
@@ -9566,6 +10476,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="10" t="inlineStr">
@@ -9617,6 +10532,11 @@
           <t>Bom Retiro</t>
         </is>
       </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="10" t="inlineStr">
@@ -9666,6 +10586,11 @@
       <c r="M187" s="10" t="inlineStr">
         <is>
           <t>Bom Retiro</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>